<commit_message>
Arreglar persistencia de correcciones ambiguos y maestro_inexacto
CAMBIOS:
- main.py (~1184): ambiguos con CONCEPTO (sin MZ) ahora usan _fuente="sin_identificar"
  → se persisten a trazabilidad Sin_identificar en lugar de perderse
  → evita que reaparezcan como pendientes al siguiente ciclo

- main.py (~1116): maestro_inexacto se persiste correctamente desde trazabilidad
  → evita redetección de pagos que ya fueron identificados con MZ-LOTE

VALIDACIÓN:
✓ Janet Vil* (S/152 + S/450) con CONCEPTO ahora persisten
✓ Identificadas en pagos_yape_tepago con estado_pago="concepto"
✓ No reaparecen en pendientes al siguiente ciclo
✓ Adolfo (I-16) sigue correcto en Maestro_inexacto sin duplicación

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_pagos/efectivo/trazabilidad/trazabilidad_2026-06.xlsx
+++ b/4_pagos/efectivo/trazabilidad/trazabilidad_2026-06.xlsx
@@ -1191,7 +1191,7 @@
         <v>4</v>
       </c>
       <c r="K9" s="15" t="n">
-        <v>46186.46313923415</v>
+        <v>46186.46313923611</v>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
@@ -1240,7 +1240,7 @@
         <v>4</v>
       </c>
       <c r="K10" s="15" t="n">
-        <v>46186.46313923415</v>
+        <v>46186.46313923611</v>
       </c>
     </row>
   </sheetData>

</xml_diff>